<commit_message>
tracking update 23.06.2026 18:22
</commit_message>
<xml_diff>
--- a/files/UAE-009_ФПЗ_07.05.2026.xlsx
+++ b/files/UAE-009_ФПЗ_07.05.2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F453691C-D85E-4996-A5DE-7160CA410AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22870777-E860-4D40-B22E-13676AE22907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2700" yWindow="2250" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э9" sheetId="1" r:id="rId1"/>
@@ -3126,6 +3126,10 @@
       <c r="Q15" s="5"/>
     </row>
     <row r="16" spans="1:1019" x14ac:dyDescent="0.2">
+      <c r="E16" s="4">
+        <f>E4-24360</f>
+        <v>984</v>
+      </c>
       <c r="K16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>

</xml_diff>

<commit_message>
tracking update 22.07.2026 22:54
</commit_message>
<xml_diff>
--- a/files/UAE-009_ФПЗ_07.05.2026.xlsx
+++ b/files/UAE-009_ФПЗ_07.05.2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#9\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#9_APMG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22870777-E860-4D40-B22E-13676AE22907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB3B8CD-6291-43F9-9579-8E7583137456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2700" yWindow="2250" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2370" yWindow="2145" windowWidth="35295" windowHeight="18060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ФПЗ_Э9" sheetId="1" r:id="rId1"/>
@@ -1850,26 +1850,25 @@
         <v>1</v>
       </c>
       <c r="E2" s="26">
-        <f>576*44</f>
-        <v>25344</v>
+        <v>24360</v>
       </c>
       <c r="F2" s="26">
         <v>12</v>
       </c>
       <c r="G2" s="26">
         <f t="shared" ref="G2" si="0">E2/F2</f>
-        <v>2112</v>
+        <v>2030</v>
       </c>
       <c r="H2" s="27">
         <v>5.9</v>
       </c>
       <c r="I2" s="27">
         <f t="shared" ref="I2" si="1">H2*E2</f>
-        <v>149529.60000000001</v>
+        <v>143724</v>
       </c>
       <c r="J2" s="28">
         <f>D2*E2*0.97</f>
-        <v>24583.68</v>
+        <v>23629.200000000001</v>
       </c>
       <c r="K2" s="24">
         <v>77.105199999999996</v>
@@ -1880,15 +1879,15 @@
       </c>
       <c r="M2" s="29">
         <f>$M$6/$I$4*I2</f>
-        <v>11529509.713919999</v>
+        <v>11081867.764799999</v>
       </c>
       <c r="N2" s="29">
         <f>$N$6/$I$4*I2</f>
-        <v>3458852.9141759998</v>
+        <v>3324560.3294399995</v>
       </c>
       <c r="O2" s="29">
         <f>$O$6/$J$4*J2</f>
-        <v>1798611.1111111112</v>
+        <v>1798611.111111111</v>
       </c>
       <c r="P2" s="29">
         <f>$P$6/$J$4*J2</f>
@@ -1896,26 +1895,26 @@
       </c>
       <c r="Q2" s="29">
         <f t="shared" ref="Q2" si="3">M2+N2+O2+P2</f>
-        <v>16810307.072540443</v>
+        <v>16228372.538684445</v>
       </c>
       <c r="R2" s="30">
         <f>SUM(Q2/E2)</f>
-        <v>663.28547476879908</v>
+        <v>666.18934887867181</v>
       </c>
       <c r="S2" s="31">
         <v>815</v>
       </c>
       <c r="T2" s="32">
         <f>(S2-R2)/R2</f>
-        <v>0.2287318673518125</v>
+        <v>0.22337590862388584</v>
       </c>
       <c r="U2" s="33">
         <f>S2*E2</f>
-        <v>20655360</v>
+        <v>19853400</v>
       </c>
       <c r="V2" s="33">
         <f t="shared" ref="V2" si="4">R2*E2</f>
-        <v>16810307.072540443</v>
+        <v>16228372.538684445</v>
       </c>
       <c r="W2" s="21"/>
       <c r="X2" s="21"/>
@@ -2938,11 +2937,11 @@
       <c r="T3" s="21"/>
       <c r="U3" s="41">
         <f>SUM(U2:U2)</f>
-        <v>20655360</v>
+        <v>19853400</v>
       </c>
       <c r="V3" s="41">
         <f>SUM(V2:V2)</f>
-        <v>16810307.072540443</v>
+        <v>16228372.538684445</v>
       </c>
       <c r="W3" s="21"/>
       <c r="X3" s="21"/>
@@ -2955,34 +2954,34 @@
       <c r="D4" s="36"/>
       <c r="E4" s="42">
         <f>SUM(E2:E3)</f>
-        <v>25344</v>
+        <v>24360</v>
       </c>
       <c r="F4" s="43"/>
       <c r="G4" s="42">
         <f>SUM(G2:G3)</f>
-        <v>2112</v>
+        <v>2030</v>
       </c>
       <c r="H4" s="43"/>
       <c r="I4" s="44">
         <f>SUMIF(I2:I2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>149529.60000000001</v>
+        <v>143724</v>
       </c>
       <c r="J4" s="45">
         <f>((SUM(J2:J2)/700)*20)+(SUM(J2:J2))</f>
-        <v>25286.070857142859</v>
+        <v>24304.32</v>
       </c>
       <c r="L4" s="7"/>
       <c r="M4" s="46">
         <f>SUMIF(M2:M2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>11529509.713919999</v>
+        <v>11081867.764799999</v>
       </c>
       <c r="N4" s="46">
         <f>SUMIF(N2:N2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>3458852.9141759998</v>
+        <v>3324560.3294399995</v>
       </c>
       <c r="O4" s="46">
         <f>SUMIF(O2:O2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>1798611.1111111112</v>
+        <v>1798611.111111111</v>
       </c>
       <c r="P4" s="46">
         <f>SUMIF(P2:P2,"&lt;&gt;#ДЕЛ/0!")</f>
@@ -2990,7 +2989,7 @@
       </c>
       <c r="Q4" s="46">
         <f>SUMIF(Q2:Q2,"&lt;&gt;#ДЕЛ/0!")</f>
-        <v>16810307.072540443</v>
+        <v>16228372.538684445</v>
       </c>
       <c r="R4" s="47"/>
       <c r="S4" s="21"/>
@@ -3023,7 +3022,7 @@
       </c>
       <c r="V5" s="51">
         <f>(U3-V3)/V3</f>
-        <v>0.22873186735181253</v>
+        <v>0.2233759086238859</v>
       </c>
     </row>
     <row r="6" spans="1:1019" ht="15.75" x14ac:dyDescent="0.25">
@@ -3031,11 +3030,11 @@
       <c r="J6" s="6"/>
       <c r="M6" s="52">
         <f>I4*K2</f>
-        <v>11529509.713919999</v>
+        <v>11081867.764799999</v>
       </c>
       <c r="N6" s="53">
         <f>M6*0.3</f>
-        <v>3458852.9141759998</v>
+        <v>3324560.3294399995</v>
       </c>
       <c r="O6" s="54">
         <v>1850000</v>
@@ -3045,11 +3044,11 @@
       </c>
       <c r="Q6" s="52">
         <f>M6+N6+O6+P6</f>
-        <v>16862362.628095999</v>
+        <v>16280428.094239999</v>
       </c>
       <c r="U6" s="41">
         <f>U3-V3</f>
-        <v>3845052.9274595566</v>
+        <v>3625027.4613155555</v>
       </c>
     </row>
     <row r="7" spans="1:1019" x14ac:dyDescent="0.2">
@@ -3128,7 +3127,7 @@
     <row r="16" spans="1:1019" x14ac:dyDescent="0.2">
       <c r="E16" s="4">
         <f>E4-24360</f>
-        <v>984</v>
+        <v>0</v>
       </c>
       <c r="K16" s="5"/>
       <c r="N16" s="5"/>

</xml_diff>